<commit_message>
Add 2 terms to Intervention content and delivery.xlsx
</commit_message>
<xml_diff>
--- a/Intervention content and delivery/Intervention content and delivery.xlsx
+++ b/Intervention content and delivery/Intervention content and delivery.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W43"/>
+  <dimension ref="A1:W45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,242 +852,233 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GMHO:0000273</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>cognitive bias modification intervention</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An intervention content that uses tasks to assess and modify a person’s cognitive bias dispositions. </t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr"/>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>LSR 6</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000122</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>A study arm designation as a comparator to some intervention arm.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>study arm</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>LSR 1; LSR 2</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="n"/>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="U8" s="2" t="n"/>
+      <c r="V8" s="2" t="n"/>
+      <c r="W8" s="2" t="inlineStr">
         <is>
           <t>PS; MS</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000177</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>daily dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Dose of pharmacological substance delivered to individuals within each day.</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
+      <c r="N9" s="3" t="n"/>
+      <c r="O9" s="3" t="n"/>
+      <c r="P9" s="3" t="n"/>
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="R9" s="3" t="n"/>
+      <c r="S9" s="3" t="n"/>
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U8" s="3" t="n"/>
-      <c r="V8" s="3" t="n"/>
-      <c r="W8" s="3" t="inlineStr">
+      <c r="U9" s="3" t="n"/>
+      <c r="V9" s="3" t="n"/>
+      <c r="W9" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>IAO:0000027</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>An information content entity that is intended to be a truthful statement about something (modulo, e.g., measurement precision or other systematic errors) and is constructed/acquired by a method which reliably tends to produce (approximately) truthful statements.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000001</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>dose of pharmacological substance</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Dose of pharmacological substance delivered to an individual.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>intervention dose</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parent class from Ontology for Biomedical Investigations
-</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1; LSR 3</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U10" s="2" t="n"/>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W10" s="2" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000265</t>
+          <t>GMHO:0000001</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>dose of physical activity intervention</t>
+          <t>dose of pharmacological substance</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Dose of physical activity intervention delivered to an individual.</t>
+          <t>Dose of pharmacological substance delivered to an individual.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1094,12 +1091,13 @@
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parent class from Ontology for Biomedical Investigations
+</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
@@ -1107,10 +1105,14 @@
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R11" s="2" t="n"/>
+          <t>LSR 1; LSR 3</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
@@ -1118,89 +1120,89 @@
         </is>
       </c>
       <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="n"/>
-      <c r="W11" s="2" t="n"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000002</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>drug name</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A written name intended to identify a particular drug. </t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>written name</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>LSR 2; LSR 3</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U12" s="3" t="n"/>
-      <c r="V12" s="3" t="inlineStr">
-        <is>
-          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W12" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000265</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>dose of physical activity intervention</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Dose of physical activity intervention delivered to an individual.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>intervention dose</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="n"/>
+      <c r="V12" s="2" t="n"/>
+      <c r="W12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000003</t>
+          <t>GMHO:0000002</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>frequency of pharmacological substance dose</t>
+          <t>drug name</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>A data item that is about the number of times a dose of pharmacological substance is delivered during an intervention.</t>
+          <t xml:space="preserve">A written name intended to identify a particular drug. </t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>written name</t>
         </is>
       </c>
       <c r="E13" s="3" t="n"/>
@@ -1217,7 +1219,7 @@
       <c r="P13" s="3" t="n"/>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>LSR 3</t>
+          <t>LSR 2; LSR 3</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
@@ -1246,22 +1248,22 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>BCIO:037000</t>
+          <t>GMHO:0000003</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>intervention</t>
+          <t>frequency of pharmacological substance dose</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>A planned process that has the aim of influencing an outcome.</t>
+          <t>A data item that is about the number of times a dose of pharmacological substance is delivered during an intervention.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E14" s="3" t="n"/>
@@ -1269,11 +1271,7 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
+      <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="n"/>
@@ -1282,10 +1280,14 @@
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>LSR 1, LSR 2, LSR 3</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="n"/>
+          <t>LSR 3</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="inlineStr">
         <is>
@@ -1293,7 +1295,11 @@
         </is>
       </c>
       <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="n"/>
+      <c r="V14" s="3" t="inlineStr">
+        <is>
+          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
+        </is>
+      </c>
       <c r="W14" s="3" t="inlineStr">
         <is>
           <t>PS</t>
@@ -1303,22 +1309,22 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000123</t>
+          <t>BCIO:037000</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>intervention arm</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>A study arm that is subject to evaluation in an intervention evaluation study.</t>
+          <t>A planned process that has the aim of influencing an outcome.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>study arm</t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E15" s="3" t="n"/>
@@ -1326,7 +1332,11 @@
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
@@ -1335,14 +1345,10 @@
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>LSR 1; LSR 2</t>
-        </is>
-      </c>
-      <c r="R15" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
+          <t>LSR 1, LSR 2, LSR 3</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="n"/>
       <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="inlineStr">
         <is>
@@ -1353,29 +1359,29 @@
       <c r="V15" s="3" t="n"/>
       <c r="W15" s="3" t="inlineStr">
         <is>
-          <t>PS; MS</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000004</t>
+          <t>GMHO:0000123</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>intervention arm name</t>
+          <t>intervention arm</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A written name intended to identify a particular intervention arm. </t>
+          <t>A study arm that is subject to evaluation in an intervention evaluation study.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>written name</t>
+          <t>study arm</t>
         </is>
       </c>
       <c r="E16" s="3" t="n"/>
@@ -1392,7 +1398,7 @@
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
+          <t>LSR 1; LSR 2</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
@@ -1407,36 +1413,32 @@
         </is>
       </c>
       <c r="U16" s="3" t="n"/>
-      <c r="V16" s="3" t="inlineStr">
-        <is>
-          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
+      <c r="V16" s="3" t="n"/>
       <c r="W16" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PS; MS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000124</t>
+          <t>GMHO:0000004</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>intervention contact event duration</t>
+          <t>intervention arm name</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>A temporal interval between the start and end of an intervention contact event.</t>
+          <t xml:space="preserve">A written name intended to identify a particular intervention arm. </t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>one-dimensional temporal region</t>
+          <t>written name</t>
         </is>
       </c>
       <c r="E17" s="3" t="n"/>
@@ -1444,28 +1446,16 @@
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>inspired by BCIO:008525</t>
-        </is>
-      </c>
-      <c r="L17" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:008525</t>
-        </is>
-      </c>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3" t="n"/>
       <c r="O17" s="3" t="n"/>
       <c r="P17" s="3" t="n"/>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>LSR 2</t>
+          <t>LSR 1; LSR 2; LSR 3</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
@@ -1479,462 +1469,486 @@
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U17" s="3" t="inlineStr">
+      <c r="U17" s="3" t="n"/>
+      <c r="V17" s="3" t="inlineStr">
+        <is>
+          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
+        </is>
+      </c>
+      <c r="W17" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000124</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>intervention contact event duration</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>A temporal interval between the start and end of an intervention contact event.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>inspired by BCIO:008525</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:008525</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="n"/>
+      <c r="P18" s="3" t="n"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="n"/>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
         <is>
           <t>Review BCIO cross reference</t>
         </is>
       </c>
-      <c r="V17" s="3" t="n"/>
-      <c r="W17" s="3" t="inlineStr">
+      <c r="V18" s="3" t="n"/>
+      <c r="W18" s="3" t="inlineStr">
         <is>
           <t>PS; MS</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>BCIO:046000</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>intervention content</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t xml:space="preserve">Based on http://humanbehaviourchange.org/ontology/BCIO_007000
 </t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>http://humanbehaviourchange.org/ontology/BCIO_007000</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000242</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>intervention dose</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>An intervention attribute that is its amount.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>drug dose and number of intervention techniques (e.g., action plans, social support)</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">"Intervention dose can capture the intensity of any intervention, including social, psychological and pharmacological interventions.
 Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities ""intervention dose"" and ""intervention schedule of delivery"". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, ""intervention dose"" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose."
 </t>
         </is>
       </c>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="2" t="n"/>
-      <c r="R19" s="2" t="n"/>
-      <c r="S19" s="2" t="n"/>
-      <c r="T19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U19" s="2" t="n"/>
-      <c r="V19" s="2" t="n"/>
-      <c r="W19" s="2" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000005</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>intervention duration</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>A temporal interval between the start and end of an intervention.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">inspired by BCIO:008560
-</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:008560</t>
-        </is>
-      </c>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
-        </is>
-      </c>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
       <c r="T20" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U20" s="2" t="inlineStr">
+      <c r="U20" s="2" t="n"/>
+      <c r="V20" s="2" t="n"/>
+      <c r="W20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000005</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A temporal interval between the start and end of an intervention.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspired by BCIO:008560
+</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:008560</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2" t="n"/>
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>LSR 1; LSR 2; LSR 3</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="n"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
         <is>
           <t>Review BCIO cross reference</t>
         </is>
       </c>
-      <c r="V20" s="2" t="inlineStr">
+      <c r="V21" s="2" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities
 Link to BCIO</t>
         </is>
       </c>
-      <c r="W20" s="2" t="inlineStr">
+      <c r="W21" s="2" t="inlineStr">
         <is>
           <t>PS; MS</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000006</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>maximum dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>A maximum value of the dose of pharmacological substance delivered to individuals in a group.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>maximum observed value</t>
         </is>
       </c>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="3" t="n"/>
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="Q21" s="3" t="inlineStr">
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>LSR 3</t>
         </is>
       </c>
-      <c r="R21" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S21" s="3" t="n"/>
-      <c r="T21" s="3" t="inlineStr">
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="n"/>
+      <c r="T22" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U21" s="3" t="n"/>
-      <c r="V21" s="3" t="inlineStr">
+      <c r="U22" s="3" t="n"/>
+      <c r="V22" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
         </is>
       </c>
-      <c r="W21" s="3" t="inlineStr">
+      <c r="W22" s="3" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>STATO:0000151</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>maximum observed value</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>A data item which denotes the largest value found in a dataset or resulting from a calculation.</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>statistic</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>LSR 3</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IAO:0000109</t>
+          <t>STATO:0000151</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>measurement datum</t>
+          <t>maximum observed value</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A measurement datum is an information content entity that is a recording of the output of a measurement such as produced by a device.</t>
+          <t>A data item which denotes the largest value found in a dataset or resulting from a calculation.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>information content entity</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
+          <t>LSR 3</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>IAO:0000109</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A measurement datum is an information content entity that is a recording of the output of a measurement such as produced by a device.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>information content entity</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>IAO:0000003</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>measurement unit label</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>A measurement unit label is as a label that is part of a scalar measurement datum and denotes a unit of measure.</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>datum label</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>LSR1; LSR2; LSR3</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000241</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention content</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>An intervention content that is part of a mental health intervention.</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>intervention content</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Any intervention content delivered in the context of a mental health intervention.</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="n"/>
-      <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="n"/>
-      <c r="T25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U25" s="2" t="n"/>
-      <c r="V25" s="2" t="n"/>
-      <c r="W25" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000260</t>
+          <t>GMHO:0000241</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario plan</t>
+          <t>mental health intervention content</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>A plan that is realized in a mental health intervention scenario process.</t>
+          <t>An intervention content that is part of a mental health intervention.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>intervention content</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Any intervention content delivered in the context of a mental health intervention.</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
@@ -1945,11 +1959,7 @@
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
+      <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="inlineStr">
@@ -1959,492 +1969,509 @@
       </c>
       <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="n"/>
-      <c r="W26" s="2" t="n"/>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000260</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>A plan that is realized in a mental health intervention scenario process.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2" t="n"/>
+      <c r="O27" s="2" t="n"/>
+      <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="2" t="n"/>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="n"/>
+      <c r="V27" s="2" t="n"/>
+      <c r="W27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000008</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>minimum dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>A minimum value of the dose of pharmacological substance delivered to individuals in a group.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>minimum value</t>
         </is>
       </c>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="n"/>
+      <c r="N28" s="3" t="n"/>
+      <c r="O28" s="3" t="n"/>
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>LSR 3</t>
         </is>
       </c>
-      <c r="R27" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S27" s="3" t="n"/>
-      <c r="T27" s="3" t="inlineStr">
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="n"/>
+      <c r="T28" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U27" s="3" t="n"/>
-      <c r="V27" s="3" t="inlineStr">
+      <c r="U28" s="3" t="n"/>
+      <c r="V28" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
         </is>
       </c>
-      <c r="W27" s="3" t="inlineStr">
+      <c r="W28" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>STATO:0000150</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>minimum observed value</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>A data item which denotes the smallest value found in a dataset or resulting from a calculation.</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>LSR 3</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000126</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>no treatment control arm</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>A control arm designation where there is no intervention.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
-      <c r="O29" s="3" t="n"/>
-      <c r="P29" s="3" t="n"/>
-      <c r="Q29" s="3" t="inlineStr">
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3" t="n"/>
+      <c r="P30" s="3" t="n"/>
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>LSR 1; LSR 2</t>
         </is>
       </c>
-      <c r="R29" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S29" s="3" t="n"/>
-      <c r="T29" s="3" t="inlineStr">
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="n"/>
+      <c r="T30" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U29" s="3" t="n"/>
-      <c r="V29" s="3" t="n"/>
-      <c r="W29" s="3" t="inlineStr">
+      <c r="U30" s="3" t="n"/>
+      <c r="V30" s="3" t="n"/>
+      <c r="W30" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>GMHO:0000274</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>number of mental health intervention contact events</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>A data item that is the number of contact events in a mental health intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr"/>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr"/>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>LSR 6</t>
+        </is>
+      </c>
+      <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S31" s="4" t="inlineStr"/>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr"/>
+      <c r="V31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>LSR 1; LSR 2; LSR 3</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="W32" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000262</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>pharmacological intervention</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Mental health intervention content that uses pharmacological substances to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>mental health intervention content</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="inlineStr">
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+      <c r="O33" s="2" t="n"/>
+      <c r="P33" s="2" t="n"/>
+      <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>LSR 1, LSR3</t>
         </is>
       </c>
-      <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="n"/>
-      <c r="T31" s="2" t="inlineStr">
+      <c r="R33" s="2" t="n"/>
+      <c r="S33" s="2" t="n"/>
+      <c r="T33" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U31" s="2" t="n"/>
-      <c r="V31" s="2" t="n"/>
-      <c r="W31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="U33" s="2" t="n"/>
+      <c r="V33" s="2" t="n"/>
+      <c r="W33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000264</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>physical activity intervention</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Mental health intervention content that uses physical performance behaviour to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>mental health intervention content</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>BCIO:036042; GMHO:0000239</t>
         </is>
       </c>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="inlineStr">
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2" t="n"/>
+      <c r="O34" s="2" t="n"/>
+      <c r="P34" s="2" t="n"/>
+      <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R32" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S32" s="2" t="n"/>
-      <c r="T32" s="2" t="inlineStr">
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="n"/>
+      <c r="T34" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U32" s="2" t="n"/>
-      <c r="V32" s="2" t="n"/>
-      <c r="W32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="U34" s="2" t="n"/>
+      <c r="V34" s="2" t="n"/>
+      <c r="W34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000194</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>physical performance behaviour pattern</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>An individual human behaviour pattern that involves repeated physical performance behaviour.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>individual human behaviour pattern</t>
         </is>
       </c>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="N33" s="3" t="n"/>
-      <c r="O33" s="3" t="n"/>
-      <c r="P33" s="3" t="n"/>
-      <c r="Q33" s="3" t="inlineStr">
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
+      <c r="M35" s="3" t="n"/>
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3" t="n"/>
+      <c r="P35" s="3" t="n"/>
+      <c r="Q35" s="3" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S33" s="3" t="n"/>
-      <c r="T33" s="3" t="inlineStr">
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S35" s="3" t="n"/>
+      <c r="T35" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U33" s="3" t="n"/>
-      <c r="V33" s="3" t="n"/>
-      <c r="W33" s="3" t="inlineStr">
+      <c r="U35" s="3" t="n"/>
+      <c r="V35" s="3" t="n"/>
+      <c r="W35" s="3" t="inlineStr">
         <is>
           <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000009</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>placebo intervention</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
-      <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="N34" s="3" t="n"/>
-      <c r="O34" s="3" t="n"/>
-      <c r="P34" s="3" t="n"/>
-      <c r="Q34" s="3" t="inlineStr">
-        <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
-        </is>
-      </c>
-      <c r="R34" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S34" s="3" t="n"/>
-      <c r="T34" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U34" s="3" t="n"/>
-      <c r="V34" s="3" t="inlineStr">
-        <is>
-          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W34" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>OBI:0000260</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>plan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000200</t>
+          <t>GMHO:0000009</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>planned pharmacological substance dose</t>
+          <t>placebo intervention</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>A plan specification about the dose of pharmacological substance.</t>
+          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>plan specification</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
@@ -2461,7 +2488,7 @@
       <c r="P36" s="3" t="n"/>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>LSR 1</t>
+          <t>LSR 1; LSR 2; LSR 3</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
@@ -2476,7 +2503,11 @@
         </is>
       </c>
       <c r="U36" s="3" t="n"/>
-      <c r="V36" s="3" t="n"/>
+      <c r="V36" s="3" t="inlineStr">
+        <is>
+          <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
+        </is>
+      </c>
       <c r="W36" s="3" t="inlineStr">
         <is>
           <t>PS</t>
@@ -2484,114 +2515,73 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000239</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>psychological intervention</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Mental health intervention content that uses communication or recommended tasks to assess and improve a person’s adaptive mental or behavioural functioning.</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention content</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>https://bciosearch.org/BCIO_050364</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050364</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="n"/>
-      <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="n"/>
-      <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="inlineStr">
-        <is>
-          <t>LSR 2</t>
-        </is>
-      </c>
-      <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="n"/>
-      <c r="T37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U37" s="2" t="n"/>
-      <c r="V37" s="2" t="n"/>
-      <c r="W37" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>OBI:0000260</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>External</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000195</t>
+          <t>GMHO:0000200</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>resistance training behaviour</t>
+          <t>planned pharmacological substance dose</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
+          <t>A plan specification about the dose of pharmacological substance.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>physical performance behaviour pattern</t>
+          <t>plan specification</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>resistance training, strength training</t>
-        </is>
-      </c>
+      <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
-        </is>
-      </c>
-      <c r="L38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> COPPER:1005</t>
-        </is>
-      </c>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
       <c r="O38" s="3" t="n"/>
       <c r="P38" s="3" t="n"/>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>LSR 2</t>
+          <t>LSR 1</t>
         </is>
       </c>
       <c r="R38" s="3" t="inlineStr">
@@ -2609,289 +2599,419 @@
       <c r="V38" s="3" t="n"/>
       <c r="W38" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000239</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>psychological intervention</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Mental health intervention content that uses communication or recommended tasks to assess and improve a person’s adaptive mental or behavioural functioning.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention content</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>https://bciosearch.org/BCIO_050364</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050364</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="n"/>
+      <c r="N39" s="2" t="n"/>
+      <c r="O39" s="2" t="n"/>
+      <c r="P39" s="2" t="n"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="n"/>
+      <c r="S39" s="2" t="n"/>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="n"/>
+      <c r="V39" s="2" t="n"/>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000195</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>resistance training behaviour</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>physical performance behaviour pattern</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>resistance training, strength training</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> COPPER:1005</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
+      <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n"/>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="n"/>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="U40" s="3" t="n"/>
+      <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="inlineStr">
+        <is>
           <t>PS; MS</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000196</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>A locomotive behaviour that involves moving at a steady pace and speed with long strides such that there is a phase at which all limbs are above the ground.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>locomotive behaviour</t>
         </is>
       </c>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>"Rubenson, J., Heliams, D. B., Lloyd, D. G., and Fournier, P. A. (2004). Gait selection in the ostrich: mechanical and metabolic characteristics of walking and running with and without an aerial phase. Proceedings of the Royal Society of London. Series B: Biological Sciences, 271(1543), 1091-1099.
 Also drew on:
 - COPPER:1011"</t>
         </is>
       </c>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
-      <c r="Q39" s="3" t="inlineStr">
+      <c r="L41" s="3" t="n"/>
+      <c r="M41" s="3" t="n"/>
+      <c r="N41" s="3" t="n"/>
+      <c r="O41" s="3" t="n"/>
+      <c r="P41" s="3" t="n"/>
+      <c r="Q41" s="3" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R39" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S39" s="3" t="n"/>
-      <c r="T39" s="3" t="inlineStr">
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="n"/>
+      <c r="T41" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U39" s="3" t="n"/>
-      <c r="V39" s="3" t="n"/>
-      <c r="W39" s="3" t="inlineStr">
+      <c r="U41" s="3" t="n"/>
+      <c r="V41" s="3" t="n"/>
+      <c r="W41" s="3" t="inlineStr">
         <is>
           <t>PS; MS</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>STATO:0000039</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>a statistic is a measurement datum to describe a dataset or a variable. It is generated by a calculation on set of observed data.</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="W42" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000127</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>study arm</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
-      <c r="J41" s="2" t="n"/>
-      <c r="K41" s="2" t="n"/>
-      <c r="L41" s="2" t="n"/>
-      <c r="M41" s="2" t="n"/>
-      <c r="N41" s="2" t="n"/>
-      <c r="O41" s="2" t="n"/>
-      <c r="P41" s="2" t="n"/>
-      <c r="Q41" s="2" t="inlineStr">
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="n"/>
+      <c r="N43" s="2" t="n"/>
+      <c r="O43" s="2" t="n"/>
+      <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R41" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S41" s="2" t="n"/>
-      <c r="T41" s="2" t="inlineStr">
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U41" s="2" t="n"/>
-      <c r="V41" s="2" t="n"/>
-      <c r="W41" s="2" t="inlineStr">
+      <c r="U43" s="2" t="n"/>
+      <c r="V43" s="2" t="n"/>
+      <c r="W43" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000128</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>treatment as usual control arm</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>A control arm designation where the same content and delivery is already provided as standard practice.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
-      <c r="J42" s="2" t="n"/>
-      <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="n"/>
-      <c r="N42" s="2" t="n"/>
-      <c r="O42" s="2" t="n"/>
-      <c r="P42" s="2" t="n"/>
-      <c r="Q42" s="2" t="inlineStr">
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="n"/>
+      <c r="M44" s="2" t="n"/>
+      <c r="N44" s="2" t="n"/>
+      <c r="O44" s="2" t="n"/>
+      <c r="P44" s="2" t="n"/>
+      <c r="Q44" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R42" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S42" s="2" t="n"/>
-      <c r="T42" s="2" t="inlineStr">
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="n"/>
+      <c r="T44" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U42" s="2" t="n"/>
-      <c r="V42" s="2" t="inlineStr">
+      <c r="U44" s="2" t="n"/>
+      <c r="V44" s="2" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>
       </c>
-      <c r="W42" s="2" t="inlineStr">
+      <c r="W44" s="2" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000129</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>waitlist control arm</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>A control arm designation where no intervention prior to the primary outcome follow-up point is delivered but participants in the study arm are informed that they will be entitled to receive an intervention at some time after that point.</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="n"/>
-      <c r="L43" s="3" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="N43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
-      <c r="P43" s="3" t="n"/>
-      <c r="Q43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
+      <c r="I45" s="3" t="n"/>
+      <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
+      <c r="L45" s="3" t="n"/>
+      <c r="M45" s="3" t="n"/>
+      <c r="N45" s="3" t="n"/>
+      <c r="O45" s="3" t="n"/>
+      <c r="P45" s="3" t="n"/>
+      <c r="Q45" s="3" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R43" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S43" s="3" t="n"/>
-      <c r="T43" s="3" t="inlineStr">
+      <c r="R45" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S45" s="3" t="n"/>
+      <c r="T45" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U43" s="3" t="n"/>
-      <c r="V43" s="3" t="inlineStr">
+      <c r="U45" s="3" t="n"/>
+      <c r="V45" s="3" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>
       </c>
-      <c r="W43" s="3" t="n"/>
+      <c r="W45" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Edit Intervention content and delivery.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/Intervention content and delivery/Intervention content and delivery.xlsx
+++ b/Intervention content and delivery/Intervention content and delivery.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W45"/>
+  <dimension ref="A1:W46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,67 +492,67 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Curator note</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Definition source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Cross reference</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'part of'</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Informal label for repository</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'part of'</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'is about'</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>LSR no.</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Ontology section</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>REL 'has part'</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'is about'</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>LSR no.</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Ontology section</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Curator note</t>
-        </is>
-      </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>To be reviewed by</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
         </is>
       </c>
     </row>
@@ -587,12 +587,12 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Based on https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6858509/</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
@@ -602,16 +602,16 @@
       <c r="S2" s="2" t="n"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="n"/>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
+      <c r="W2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -667,18 +667,18 @@
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="V3" s="3" t="n"/>
+      <c r="W3" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -720,12 +720,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -756,12 +756,12 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Insipred by https://www.merriam-webster.com/dictionary/bodybuilding</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
@@ -771,16 +771,16 @@
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
-      <c r="W5" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="W5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -813,17 +813,17 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Cross-reference: COPPER:1044 - changed parent class</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>COPPER:1044</t>
         </is>
       </c>
-      <c r="M6" s="3" t="n"/>
       <c r="N6" s="3" t="n"/>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="n"/>
@@ -840,16 +840,16 @@
       <c r="S6" s="3" t="n"/>
       <c r="T6" s="3" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U6" s="3" t="n"/>
       <c r="V6" s="3" t="n"/>
-      <c r="W6" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="W6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -872,22 +872,22 @@
           <t>intervention content</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Intervention content and delivery</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>LSR 6</t>
@@ -898,15 +898,15 @@
           <t>Intervention content and delivery</t>
         </is>
       </c>
-      <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr">
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="4" t="n"/>
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr"/>
-      <c r="V7" s="4" t="inlineStr"/>
-      <c r="W7" s="4" t="inlineStr"/>
+      <c r="V7" s="4" t="n"/>
+      <c r="W7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -954,16 +954,16 @@
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="2" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U8" s="2" t="n"/>
       <c r="V8" s="2" t="n"/>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="W8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1007,16 +1007,16 @@
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U9" s="3" t="n"/>
       <c r="V9" s="3" t="n"/>
-      <c r="W9" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="W9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -1092,13 +1092,13 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Parent class from Ontology for Biomedical Investigations
 </t>
         </is>
       </c>
-      <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
@@ -1116,18 +1116,18 @@
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="inlineStr">
+      <c r="V11" s="2" t="n"/>
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W11" s="2" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
-      <c r="T12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="n"/>
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U12" s="2" t="n"/>
       <c r="V12" s="2" t="n"/>
       <c r="W12" s="2" t="n"/>
     </row>
@@ -1230,18 +1230,18 @@
       <c r="S13" s="3" t="n"/>
       <c r="T13" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U13" s="3" t="n"/>
-      <c r="V13" s="3" t="inlineStr">
+      <c r="V13" s="3" t="n"/>
+      <c r="W13" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W13" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -1291,18 +1291,18 @@
       <c r="S14" s="3" t="n"/>
       <c r="T14" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="inlineStr">
+      <c r="V14" s="3" t="n"/>
+      <c r="W14" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W14" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -1352,16 +1352,16 @@
       <c r="S15" s="3" t="n"/>
       <c r="T15" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U15" s="3" t="n"/>
       <c r="V15" s="3" t="n"/>
-      <c r="W15" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="W15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1409,16 +1409,16 @@
       <c r="S16" s="3" t="n"/>
       <c r="T16" s="3" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U16" s="3" t="n"/>
       <c r="V16" s="3" t="n"/>
-      <c r="W16" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="W16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1466,18 +1466,18 @@
       <c r="S17" s="3" t="n"/>
       <c r="T17" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U17" s="3" t="n"/>
-      <c r="V17" s="3" t="inlineStr">
+      <c r="V17" s="3" t="n"/>
+      <c r="W17" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W17" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
@@ -1512,17 +1512,17 @@
           <t>intervention content and delivery</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>inspired by BCIO:008525</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>BCIO:008525</t>
         </is>
       </c>
-      <c r="M18" s="3" t="n"/>
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="n"/>
       <c r="P18" s="3" t="n"/>
@@ -1539,20 +1539,20 @@
       <c r="S18" s="3" t="n"/>
       <c r="T18" s="3" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U18" s="3" t="inlineStr">
+      <c r="V18" s="3" t="inlineStr">
         <is>
           <t>Review BCIO cross reference</t>
         </is>
       </c>
-      <c r="V18" s="3" t="n"/>
-      <c r="W18" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="W18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1575,13 +1575,13 @@
           <t>planned process</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t xml:space="preserve">Based on http://humanbehaviourchange.org/ontology/BCIO_007000
 </t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>http://humanbehaviourchange.org/ontology/BCIO_007000</t>
         </is>
@@ -1598,12 +1598,12 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>MS</t>
         </is>
       </c>
     </row>
@@ -1653,351 +1653,351 @@
       <c r="Q20" s="2" t="n"/>
       <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="inlineStr">
+      <c r="T20" s="2" t="n"/>
+      <c r="U20" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U20" s="2" t="n"/>
       <c r="V20" s="2" t="n"/>
       <c r="W20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000005</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>intervention duration</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>A temporal interval between the start and end of an intervention.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>intervention content and delivery</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">inspired by BCIO:008560
 </t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>BCIO:008560</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="inlineStr">
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="n"/>
+      <c r="P21" s="3" t="n"/>
+      <c r="Q21" s="3" t="inlineStr">
         <is>
           <t>LSR 1; LSR 2; LSR 3</t>
         </is>
       </c>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="n"/>
-      <c r="T21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U21" s="2" t="inlineStr">
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="n"/>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="inlineStr">
         <is>
           <t>Review BCIO cross reference</t>
         </is>
       </c>
-      <c r="V21" s="2" t="inlineStr">
+      <c r="W21" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities
 Link to BCIO</t>
         </is>
       </c>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BCIO:008560</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>intervention duration</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A &lt;temporal interval&gt; between the start and end of an intervention.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>The planned duration of an intervention</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000006</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>maximum dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>A maximum value of the dose of pharmacological substance delivered to individuals in a group.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>maximum observed value</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3" t="n"/>
+      <c r="P23" s="3" t="inlineStr">
         <is>
           <t>dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>LSR 3</t>
         </is>
       </c>
-      <c r="R22" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S22" s="3" t="n"/>
-      <c r="T22" s="3" t="inlineStr">
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="n"/>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U22" s="3" t="n"/>
-      <c r="V22" s="3" t="inlineStr">
+      <c r="V23" s="3" t="n"/>
+      <c r="W23" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
-        </is>
-      </c>
-      <c r="W22" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>STATO:0000151</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>maximum observed value</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>A data item which denotes the largest value found in a dataset or resulting from a calculation.</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>statistic</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>LSR 3</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IAO:0000109</t>
+          <t>STATO:0000151</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>measurement datum</t>
+          <t>maximum observed value</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A measurement datum is an information content entity that is a recording of the output of a measurement such as produced by a device.</t>
+          <t>A data item which denotes the largest value found in a dataset or resulting from a calculation.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>information content entity</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
+          <t>LSR 3</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>IAO:0000109</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A measurement datum is an information content entity that is a recording of the output of a measurement such as produced by a device.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>information content entity</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>IAO:0000003</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>measurement unit label</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>A measurement unit label is as a label that is part of a scalar measurement datum and denotes a unit of measure.</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>datum label</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>LSR1; LSR2; LSR3</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000241</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention content</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>An intervention content that is part of a mental health intervention.</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>intervention content</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Any intervention content delivered in the context of a mental health intervention.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="n"/>
-      <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="n"/>
-      <c r="T26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U26" s="2" t="n"/>
-      <c r="V26" s="2" t="n"/>
-      <c r="W26" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000260</t>
+          <t>GMHO:0000241</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario plan</t>
+          <t>mental health intervention content</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>A plan that is realized in a mental health intervention scenario process.</t>
+          <t>An intervention content that is part of a mental health intervention.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>intervention content</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Any intervention content delivered in the context of a mental health intervention.</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
@@ -2008,347 +2008,343 @@
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
+      <c r="Q27" s="2" t="n"/>
       <c r="R27" s="2" t="n"/>
       <c r="S27" s="2" t="n"/>
       <c r="T27" s="2" t="inlineStr">
         <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U27" s="2" t="n"/>
       <c r="V27" s="2" t="n"/>
       <c r="W27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000260</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>A plan that is realized in a mental health intervention scenario process.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="n"/>
+      <c r="O28" s="2" t="n"/>
+      <c r="P28" s="2" t="n"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="2" t="n"/>
+      <c r="T28" s="2" t="n"/>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="n"/>
+      <c r="W28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000008</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>minimum dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>A minimum value of the dose of pharmacological substance delivered to individuals in a group.</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>minimum value</t>
         </is>
       </c>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
+      <c r="M29" s="3" t="n"/>
+      <c r="N29" s="3" t="n"/>
+      <c r="O29" s="3" t="n"/>
+      <c r="P29" s="3" t="inlineStr">
         <is>
           <t>dose of pharmacological substance</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
+      <c r="Q29" s="3" t="inlineStr">
         <is>
           <t>LSR 3</t>
         </is>
       </c>
-      <c r="R28" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S28" s="3" t="n"/>
-      <c r="T28" s="3" t="inlineStr">
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="n"/>
+      <c r="T29" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U29" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U28" s="3" t="n"/>
-      <c r="V28" s="3" t="inlineStr">
+      <c r="V29" s="3" t="n"/>
+      <c r="W29" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
         </is>
       </c>
-      <c r="W28" s="3" t="inlineStr">
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>STATO:0000150</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>minimum observed value</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A data item which denotes the smallest value found in a dataset or resulting from a calculation.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>statistic</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>LSR 3</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000126</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>no treatment control arm</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>A control arm designation where there is no intervention.</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>control arm</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="3" t="n"/>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
+      <c r="M31" s="3" t="n"/>
+      <c r="N31" s="3" t="n"/>
+      <c r="O31" s="3" t="n"/>
+      <c r="P31" s="3" t="n"/>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>LSR 1; LSR 2</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S31" s="3" t="n"/>
+      <c r="T31" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>STATO:0000150</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>minimum observed value</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>A data item which denotes the smallest value found in a dataset or resulting from a calculation.</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>statistic</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>LSR 3</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
+      <c r="U31" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V31" s="3" t="n"/>
+      <c r="W31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>GMHO:0000274</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>number of mental health intervention contact events</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>A data item that is the number of contact events in a mental health intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="n"/>
+      <c r="O32" s="4" t="n"/>
+      <c r="P32" s="4" t="n"/>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>LSR 6</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S32" s="4" t="n"/>
+      <c r="T32" s="4" t="n"/>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="n"/>
+      <c r="W32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BFO:0000038</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>one-dimensional temporal region</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>A one-dimensional temporal region is a temporal region that is extended.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>temporal region</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>LSR 1; LSR 2; LSR 3</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000126</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>no treatment control arm</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>A control arm designation where there is no intervention.</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>control arm</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3" t="n"/>
-      <c r="P30" s="3" t="n"/>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>LSR 1; LSR 2</t>
-        </is>
-      </c>
-      <c r="R30" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S30" s="3" t="n"/>
-      <c r="T30" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U30" s="3" t="n"/>
-      <c r="V30" s="3" t="n"/>
-      <c r="W30" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>GMHO:0000274</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>number of mental health intervention contact events</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>A data item that is the number of contact events in a mental health intervention temporal part.</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
-      <c r="Q31" s="4" t="inlineStr">
-        <is>
-          <t>LSR 6</t>
-        </is>
-      </c>
-      <c r="R31" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S31" s="4" t="inlineStr"/>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="inlineStr"/>
-      <c r="V31" s="4" t="inlineStr"/>
-      <c r="W31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>BFO:0000038</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>one-dimensional temporal region</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>A one-dimensional temporal region is a temporal region that is extended.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>temporal region</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000262</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>pharmacological intervention</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Mental health intervention content that uses pharmacological substances to assess and improve a person’s adaptive mental or behavioural functioning.</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention content</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="n"/>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1, LSR3</t>
-        </is>
-      </c>
-      <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="n"/>
-      <c r="T33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U33" s="2" t="n"/>
-      <c r="V33" s="2" t="n"/>
-      <c r="W33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000264</t>
+          <t>GMHO:0000262</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>physical activity intervention</t>
+          <t>pharmacological intervention</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mental health intervention content that uses physical performance behaviour to assess and improve a person’s adaptive mental or behavioural functioning.</t>
+          <t>Mental health intervention content that uses pharmacological substances to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2366,11 +2362,7 @@
           <t>Intervention content and delivery</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:036042; GMHO:0000239</t>
-        </is>
-      </c>
+      <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
@@ -2378,100 +2370,100 @@
       <c r="P34" s="2" t="n"/>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>LSR 2</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
+          <t>LSR 1, LSR3</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="n"/>
       <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="inlineStr">
+      <c r="T34" s="2" t="n"/>
+      <c r="U34" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U34" s="2" t="n"/>
       <c r="V34" s="2" t="n"/>
       <c r="W34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000194</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>physical performance behaviour pattern</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>An individual human behaviour pattern that involves repeated physical performance behaviour.</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>individual human behaviour pattern</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3" t="n"/>
-      <c r="O35" s="3" t="n"/>
-      <c r="P35" s="3" t="n"/>
-      <c r="Q35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000264</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>physical activity intervention</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Mental health intervention content that uses physical performance behaviour to assess and improve a person’s adaptive mental or behavioural functioning.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention content</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:036042; GMHO:0000239</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="2" t="n"/>
+      <c r="P35" s="2" t="n"/>
+      <c r="Q35" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S35" s="3" t="n"/>
-      <c r="T35" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U35" s="3" t="n"/>
-      <c r="V35" s="3" t="n"/>
-      <c r="W35" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S35" s="2" t="n"/>
+      <c r="T35" s="2" t="n"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="n"/>
+      <c r="W35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000009</t>
+          <t>GMHO:0000194</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>placebo intervention</t>
+          <t>physical performance behaviour pattern</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
+          <t>An individual human behaviour pattern that involves repeated physical performance behaviour.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>intervention</t>
+          <t>individual human behaviour pattern</t>
         </is>
       </c>
       <c r="E36" s="3" t="n"/>
@@ -2488,7 +2480,7 @@
       <c r="P36" s="3" t="n"/>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
+          <t>LSR 2</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
@@ -2499,276 +2491,270 @@
       <c r="S36" s="3" t="n"/>
       <c r="T36" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U36" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U36" s="3" t="n"/>
-      <c r="V36" s="3" t="inlineStr">
+      <c r="V36" s="3" t="n"/>
+      <c r="W36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000009</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>placebo intervention</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="n"/>
+      <c r="N37" s="3" t="n"/>
+      <c r="O37" s="3" t="n"/>
+      <c r="P37" s="3" t="n"/>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>LSR 1; LSR 2; LSR 3</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="n"/>
+      <c r="T37" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U37" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V37" s="3" t="n"/>
+      <c r="W37" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
         </is>
       </c>
-      <c r="W36" s="3" t="inlineStr">
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>OBI:0000260</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000200</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>planned pharmacological substance dose</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>A plan specification about the dose of pharmacological substance.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>plan specification</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="3" t="n"/>
+      <c r="N39" s="3" t="n"/>
+      <c r="O39" s="3" t="n"/>
+      <c r="P39" s="3" t="n"/>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>LSR 1</t>
+        </is>
+      </c>
+      <c r="R39" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S39" s="3" t="n"/>
+      <c r="T39" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>OBI:0000260</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>plan</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000200</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>planned pharmacological substance dose</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>A plan specification about the dose of pharmacological substance.</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>plan specification</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="n"/>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="N38" s="3" t="n"/>
-      <c r="O38" s="3" t="n"/>
-      <c r="P38" s="3" t="n"/>
-      <c r="Q38" s="3" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="R38" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S38" s="3" t="n"/>
-      <c r="T38" s="3" t="inlineStr">
+      <c r="U39" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U38" s="3" t="n"/>
-      <c r="V38" s="3" t="n"/>
-      <c r="W38" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="V39" s="3" t="n"/>
+      <c r="W39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000239</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>psychological intervention</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Mental health intervention content that uses communication or recommended tasks to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>mental health intervention content</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>https://bciosearch.org/BCIO_050364</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>BCIO:050364</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n"/>
-      <c r="N39" s="2" t="n"/>
-      <c r="O39" s="2" t="n"/>
-      <c r="P39" s="2" t="n"/>
-      <c r="Q39" s="2" t="inlineStr">
+      <c r="N40" s="2" t="n"/>
+      <c r="O40" s="2" t="n"/>
+      <c r="P40" s="2" t="n"/>
+      <c r="Q40" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R39" s="2" t="n"/>
-      <c r="S39" s="2" t="n"/>
-      <c r="T39" s="2" t="inlineStr">
+      <c r="R40" s="2" t="n"/>
+      <c r="S40" s="2" t="n"/>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U39" s="2" t="n"/>
-      <c r="V39" s="2" t="n"/>
-      <c r="W39" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000195</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>resistance training behaviour</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>physical performance behaviour pattern</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>resistance training, strength training</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
-        </is>
-      </c>
-      <c r="L40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> COPPER:1005</t>
-        </is>
-      </c>
-      <c r="M40" s="3" t="n"/>
-      <c r="N40" s="3" t="n"/>
-      <c r="O40" s="3" t="n"/>
-      <c r="P40" s="3" t="n"/>
-      <c r="Q40" s="3" t="inlineStr">
-        <is>
-          <t>LSR 2</t>
-        </is>
-      </c>
-      <c r="R40" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S40" s="3" t="n"/>
-      <c r="T40" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U40" s="3" t="n"/>
-      <c r="V40" s="3" t="n"/>
-      <c r="W40" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
+      <c r="V40" s="2" t="n"/>
+      <c r="W40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000196</t>
+          <t>GMHO:0000195</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>resistance training behaviour</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>A locomotive behaviour that involves moving at a steady pace and speed with long strides such that there is a phase at which all limbs are above the ground.</t>
+          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>locomotive behaviour</t>
+          <t>physical performance behaviour pattern</t>
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>resistance training, strength training</t>
+        </is>
+      </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>"Rubenson, J., Heliams, D. B., Lloyd, D. G., and Fournier, P. A. (2004). Gait selection in the ostrich: mechanical and metabolic characteristics of walking and running with and without an aerial phase. Proceedings of the Royal Society of London. Series B: Biological Sciences, 271(1543), 1091-1099.
-Also drew on:
-- COPPER:1011"</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="n"/>
-      <c r="M41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> COPPER:1005</t>
+        </is>
+      </c>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
       <c r="P41" s="3" t="n"/>
@@ -2785,135 +2771,141 @@
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="inlineStr">
         <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U41" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U41" s="3" t="n"/>
       <c r="V41" s="3" t="n"/>
-      <c r="W41" s="3" t="inlineStr">
+      <c r="W41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000196</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>A locomotive behaviour that involves moving at a steady pace and speed with long strides such that there is a phase at which all limbs are above the ground.</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>locomotive behaviour</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>"Rubenson, J., Heliams, D. B., Lloyd, D. G., and Fournier, P. A. (2004). Gait selection in the ostrich: mechanical and metabolic characteristics of walking and running with and without an aerial phase. Proceedings of the Royal Society of London. Series B: Biological Sciences, 271(1543), 1091-1099.
+Also drew on:
+- COPPER:1011"</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
+      <c r="O42" s="3" t="n"/>
+      <c r="P42" s="3" t="n"/>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S42" s="3" t="n"/>
+      <c r="T42" s="3" t="inlineStr">
         <is>
           <t>PS; MS</t>
         </is>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="U42" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V42" s="3" t="n"/>
+      <c r="W42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>STATO:0000039</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>a statistic is a measurement datum to describe a dataset or a variable. It is generated by a calculation on set of observed data.</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T42" t="inlineStr">
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000127</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>study arm</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>information content entity</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
-      <c r="J43" s="2" t="n"/>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n"/>
-      <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="n"/>
-      <c r="P43" s="2" t="n"/>
-      <c r="Q43" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="R43" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S43" s="2" t="n"/>
-      <c r="T43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="U43" s="2" t="n"/>
-      <c r="V43" s="2" t="n"/>
-      <c r="W43" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000128</t>
+          <t>GMHO:0000127</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>treatment as usual control arm</t>
+          <t>study arm</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>A control arm designation where the same content and delivery is already provided as standard practice.</t>
+          <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>control arm</t>
+          <t>information content entity</t>
         </is>
       </c>
       <c r="E44" s="2" t="n"/>
@@ -2930,7 +2922,7 @@
       <c r="P44" s="2" t="n"/>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>LSR 2</t>
+          <t>LSR 1</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
@@ -2941,77 +2933,134 @@
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U44" s="2" t="n"/>
-      <c r="V44" s="2" t="inlineStr">
+      <c r="V44" s="2" t="n"/>
+      <c r="W44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000128</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>treatment as usual control arm</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>A control arm designation where the same content and delivery is already provided as standard practice.</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>control arm</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
+      <c r="M45" s="2" t="n"/>
+      <c r="N45" s="2" t="n"/>
+      <c r="O45" s="2" t="n"/>
+      <c r="P45" s="2" t="n"/>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="n"/>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="n"/>
+      <c r="W45" s="2" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>
       </c>
-      <c r="W44" s="2" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000129</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>waitlist control arm</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>A control arm designation where no intervention prior to the primary outcome follow-up point is delivered but participants in the study arm are informed that they will be entitled to receive an intervention at some time after that point.</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
-      <c r="I45" s="3" t="n"/>
-      <c r="J45" s="3" t="n"/>
-      <c r="K45" s="3" t="n"/>
-      <c r="L45" s="3" t="n"/>
-      <c r="M45" s="3" t="n"/>
-      <c r="N45" s="3" t="n"/>
-      <c r="O45" s="3" t="n"/>
-      <c r="P45" s="3" t="n"/>
-      <c r="Q45" s="3" t="inlineStr">
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
+      <c r="O46" s="3" t="n"/>
+      <c r="P46" s="3" t="n"/>
+      <c r="Q46" s="3" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R45" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S45" s="3" t="n"/>
-      <c r="T45" s="3" t="inlineStr">
+      <c r="R46" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="n"/>
+      <c r="T46" s="3" t="n"/>
+      <c r="U46" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U45" s="3" t="n"/>
-      <c r="V45" s="3" t="inlineStr">
+      <c r="V46" s="3" t="n"/>
+      <c r="W46" s="3" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>
       </c>
-      <c r="W45" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Edit Intervention content and delivery.xlsx: update 2, add 1
</commit_message>
<xml_diff>
--- a/Intervention content and delivery/Intervention content and delivery.xlsx
+++ b/Intervention content and delivery/Intervention content and delivery.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W46"/>
+  <dimension ref="A1:W47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -852,61 +846,61 @@
       <c r="W6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000273</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>cognitive bias modification intervention</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">An intervention content that uses tasks to assess and modify a person’s cognitive bias dispositions. </t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>intervention content</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>LSR 6</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="n"/>
-      <c r="W7" s="4" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="n"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="n"/>
+      <c r="W7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1762,33 +1756,16 @@
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>The planned duration of an intervention</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2228,176 +2205,172 @@
       <c r="W31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BCIO:008515</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>number of intervention contact events</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>The planned total number of sessions or digital contacts in an intervention or part</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000274</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>number of mental health intervention contact events</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>A data item that is the number of contact events in a mental health intervention temporal part.</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="n"/>
-      <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
-      <c r="O32" s="4" t="n"/>
-      <c r="P32" s="4" t="n"/>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
+      <c r="O33" s="3" t="n"/>
+      <c r="P33" s="3" t="n"/>
+      <c r="Q33" s="3" t="inlineStr">
         <is>
           <t>LSR 6</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S32" s="4" t="n"/>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="n"/>
-      <c r="W32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="n"/>
+      <c r="T33" s="3" t="n"/>
+      <c r="U33" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V33" s="3" t="n"/>
+      <c r="W33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>BFO:0000038</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>one-dimensional temporal region</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>A one-dimensional temporal region is a temporal region that is extended.</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>temporal region</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>LSR 1; LSR 2; LSR 3</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="U34" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000262</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>pharmacological intervention</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Mental health intervention content that uses pharmacological substances to assess and improve a person’s adaptive mental or behavioural functioning.</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention content</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1, LSR3</t>
-        </is>
-      </c>
-      <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="n"/>
-      <c r="U34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V34" s="2" t="n"/>
-      <c r="W34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000264</t>
+          <t>GMHO:0000262</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>physical activity intervention</t>
+          <t>pharmacological intervention</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mental health intervention content that uses physical performance behaviour to assess and improve a person’s adaptive mental or behavioural functioning.</t>
+          <t>Mental health intervention content that uses pharmacological substances to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2416,25 +2389,17 @@
         </is>
       </c>
       <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:036042; GMHO:0000239</t>
-        </is>
-      </c>
+      <c r="L35" s="2" t="n"/>
       <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>LSR 2</t>
-        </is>
-      </c>
-      <c r="R35" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
+          <t>LSR 1, LSR3</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="n"/>
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="2" t="n"/>
       <c r="U35" s="2" t="inlineStr">
@@ -2446,81 +2411,85 @@
       <c r="W35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000194</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>physical performance behaviour pattern</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>An individual human behaviour pattern that involves repeated physical performance behaviour.</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>individual human behaviour pattern</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
-      <c r="L36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="N36" s="3" t="n"/>
-      <c r="O36" s="3" t="n"/>
-      <c r="P36" s="3" t="n"/>
-      <c r="Q36" s="3" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000264</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>physical activity intervention</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Mental health intervention content that uses physical performance behaviour to assess and improve a person’s adaptive mental or behavioural functioning.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention content</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:036042; GMHO:0000239</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="n"/>
+      <c r="N36" s="2" t="n"/>
+      <c r="O36" s="2" t="n"/>
+      <c r="P36" s="2" t="n"/>
+      <c r="Q36" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R36" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S36" s="3" t="n"/>
-      <c r="T36" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U36" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="V36" s="3" t="n"/>
-      <c r="W36" s="3" t="n"/>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="n"/>
+      <c r="T36" s="2" t="n"/>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="n"/>
+      <c r="W36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000009</t>
+          <t>GMHO:0000194</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>placebo intervention</t>
+          <t>physical performance behaviour pattern</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
+          <t>An individual human behaviour pattern that involves repeated physical performance behaviour.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>intervention</t>
+          <t>individual human behaviour pattern</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
@@ -2537,7 +2506,7 @@
       <c r="P37" s="3" t="n"/>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>LSR 1; LSR 2; LSR 3</t>
+          <t>LSR 2</t>
         </is>
       </c>
       <c r="R37" s="3" t="inlineStr">
@@ -2557,267 +2526,261 @@
         </is>
       </c>
       <c r="V37" s="3" t="n"/>
-      <c r="W37" s="3" t="inlineStr">
+      <c r="W37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000009</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>placebo intervention</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>An intervention that has the same or similar appearance and delivery to another intervention but is intended not to have the active content of that intervention.</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="n"/>
+      <c r="H38" s="3" t="n"/>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="n"/>
+      <c r="N38" s="3" t="n"/>
+      <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>LSR 1; LSR 2; LSR 3</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="n"/>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U38" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V38" s="3" t="n"/>
+      <c r="W38" s="3" t="inlineStr">
         <is>
           <t>external parent class needs to be represented on Github spreadsheet for external entities</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>OBI:0000260</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>plan</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000200</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>planned pharmacological substance dose</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>A plan specification about the dose of pharmacological substance.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>plan specification</t>
         </is>
       </c>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
-      <c r="Q39" s="3" t="inlineStr">
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
+      <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n"/>
+      <c r="Q40" s="3" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R39" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S39" s="3" t="n"/>
-      <c r="T39" s="3" t="inlineStr">
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="n"/>
+      <c r="T40" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="U39" s="3" t="inlineStr">
+      <c r="U40" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="V39" s="3" t="n"/>
-      <c r="W39" s="3" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000239</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>psychological intervention</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Mental health intervention content that uses communication or recommended tasks to assess and improve a person’s adaptive mental or behavioural functioning.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>mental health intervention content</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>https://bciosearch.org/BCIO_050364</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>BCIO:050364</t>
         </is>
       </c>
-      <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
-      <c r="P40" s="2" t="n"/>
-      <c r="Q40" s="2" t="inlineStr">
+      <c r="N41" s="2" t="n"/>
+      <c r="O41" s="2" t="n"/>
+      <c r="P41" s="2" t="n"/>
+      <c r="Q41" s="2" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="n"/>
-      <c r="T40" s="2" t="inlineStr">
+      <c r="R41" s="2" t="n"/>
+      <c r="S41" s="2" t="n"/>
+      <c r="T41" s="2" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="U40" s="2" t="inlineStr">
+      <c r="U41" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="V40" s="2" t="n"/>
-      <c r="W40" s="2" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000195</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>resistance training behaviour</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>physical performance behaviour pattern</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>resistance training, strength training</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
-        </is>
-      </c>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> COPPER:1005</t>
-        </is>
-      </c>
-      <c r="N41" s="3" t="n"/>
-      <c r="O41" s="3" t="n"/>
-      <c r="P41" s="3" t="n"/>
-      <c r="Q41" s="3" t="inlineStr">
-        <is>
-          <t>LSR 2</t>
-        </is>
-      </c>
-      <c r="R41" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S41" s="3" t="n"/>
-      <c r="T41" s="3" t="inlineStr">
-        <is>
-          <t>PS; MS</t>
-        </is>
-      </c>
-      <c r="U41" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="V41" s="3" t="n"/>
-      <c r="W41" s="3" t="n"/>
+      <c r="V41" s="2" t="n"/>
+      <c r="W41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000196</t>
+          <t>GMHO:0000195</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>resistance training behaviour</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>A locomotive behaviour that involves moving at a steady pace and speed with long strides such that there is a phase at which all limbs are above the ground.</t>
+          <t>Physical performance behaviour pattern that uses weight, or other forms of resistance, to induce muscle contraction and build strength, anaerobic endurance, and size of skeletal muscles.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>locomotive behaviour</t>
+          <t>physical performance behaviour pattern</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>resistance training, strength training</t>
+        </is>
+      </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="n"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>"Rubenson, J., Heliams, D. B., Lloyd, D. G., and Fournier, P. A. (2004). Gait selection in the ostrich: mechanical and metabolic characteristics of walking and running with and without an aerial phase. Proceedings of the Royal Society of London. Series B: Biological Sciences, 271(1543), 1091-1099.
-Also drew on:
-- COPPER:1011"</t>
-        </is>
-      </c>
-      <c r="M42" s="3" t="n"/>
+          <t xml:space="preserve">Crosss-reference: COPPER:1005 - changed parent class - definition in their ontology adapted definitions from NCIT_C154219 </t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> COPPER:1005</t>
+        </is>
+      </c>
       <c r="N42" s="3" t="n"/>
       <c r="O42" s="3" t="n"/>
       <c r="P42" s="3" t="n"/>
@@ -2846,123 +2809,129 @@
       <c r="W42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000196</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>A locomotive behaviour that involves moving at a steady pace and speed with long strides such that there is a phase at which all limbs are above the ground.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>locomotive behaviour</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>"Rubenson, J., Heliams, D. B., Lloyd, D. G., and Fournier, P. A. (2004). Gait selection in the ostrich: mechanical and metabolic characteristics of walking and running with and without an aerial phase. Proceedings of the Royal Society of London. Series B: Biological Sciences, 271(1543), 1091-1099.
+Also drew on:
+- COPPER:1011"</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="n"/>
+      <c r="T43" s="3" t="inlineStr">
+        <is>
+          <t>PS; MS</t>
+        </is>
+      </c>
+      <c r="U43" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="V43" s="3" t="n"/>
+      <c r="W43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>STATO:0000039</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>statistic</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>a statistic is a measurement datum to describe a dataset or a variable. It is generated by a calculation on set of observed data.</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
+      <c r="Q44" t="inlineStr">
         <is>
           <t>LSR 1</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U44" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000127</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>study arm</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>information content entity</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="n"/>
-      <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="n"/>
-      <c r="P44" s="2" t="n"/>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>LSR 1</t>
-        </is>
-      </c>
-      <c r="R44" s="2" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S44" s="2" t="n"/>
-      <c r="T44" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="V44" s="2" t="n"/>
-      <c r="W44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000128</t>
+          <t>GMHO:0000127</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>treatment as usual control arm</t>
+          <t>study arm</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>A control arm designation where the same content and delivery is already provided as standard practice.</t>
+          <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>control arm</t>
+          <t>information content entity</t>
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
@@ -2979,7 +2948,7 @@
       <c r="P45" s="2" t="n"/>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>LSR 2</t>
+          <t>LSR 1</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -2990,73 +2959,130 @@
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="n"/>
+      <c r="W45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000128</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>treatment as usual control arm</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>A control arm designation where the same content and delivery is already provided as standard practice.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>control arm</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="n"/>
+      <c r="M46" s="2" t="n"/>
+      <c r="N46" s="2" t="n"/>
+      <c r="O46" s="2" t="n"/>
+      <c r="P46" s="2" t="n"/>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>LSR 2</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n"/>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="U45" s="2" t="inlineStr">
+      <c r="U46" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="V45" s="2" t="n"/>
-      <c r="W45" s="2" t="inlineStr">
+      <c r="V46" s="2" t="n"/>
+      <c r="W46" s="2" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000129</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>waitlist control arm</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>A control arm designation where no intervention prior to the primary outcome follow-up point is delivered but participants in the study arm are informed that they will be entitled to receive an intervention at some time after that point.</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>control arm</t>
         </is>
       </c>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="3" t="n"/>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="3" t="n"/>
-      <c r="I46" s="3" t="n"/>
-      <c r="J46" s="3" t="n"/>
-      <c r="K46" s="3" t="n"/>
-      <c r="L46" s="3" t="n"/>
-      <c r="M46" s="3" t="n"/>
-      <c r="N46" s="3" t="n"/>
-      <c r="O46" s="3" t="n"/>
-      <c r="P46" s="3" t="n"/>
-      <c r="Q46" s="3" t="inlineStr">
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
+      <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="n"/>
+      <c r="I47" s="3" t="n"/>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
+      <c r="L47" s="3" t="n"/>
+      <c r="M47" s="3" t="n"/>
+      <c r="N47" s="3" t="n"/>
+      <c r="O47" s="3" t="n"/>
+      <c r="P47" s="3" t="n"/>
+      <c r="Q47" s="3" t="inlineStr">
         <is>
           <t>LSR 2</t>
         </is>
       </c>
-      <c r="R46" s="3" t="inlineStr">
-        <is>
-          <t>Intervention content and delivery</t>
-        </is>
-      </c>
-      <c r="S46" s="3" t="n"/>
-      <c r="T46" s="3" t="n"/>
-      <c r="U46" s="3" t="inlineStr">
+      <c r="R47" s="3" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="S47" s="3" t="n"/>
+      <c r="T47" s="3" t="n"/>
+      <c r="U47" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="V46" s="3" t="n"/>
-      <c r="W46" s="3" t="inlineStr">
+      <c r="V47" s="3" t="n"/>
+      <c r="W47" s="3" t="inlineStr">
         <is>
           <t>propose to external ontology</t>
         </is>

</xml_diff>